<commit_message>
Actualizar archivo maestro modelo
</commit_message>
<xml_diff>
--- a/2. PASAJES FFVV JULIO 2026 MODELO.xlsx
+++ b/2. PASAJES FFVV JULIO 2026 MODELO.xlsx
@@ -2,31 +2,40 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alarc\OneDrive\Documentos\PROGRAMAS\PLANILLAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F024C2-2850-4E30-8DBE-E8FB1AA61872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DEAAD9D-6675-4D5D-99D5-97B867C251A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BBVA" sheetId="1" r:id="rId1"/>
     <sheet name="BCP" sheetId="2" r:id="rId2"/>
     <sheet name="SCOTIABANK" sheetId="3" r:id="rId3"/>
     <sheet name="FINANCIERO" sheetId="4" r:id="rId4"/>
-    <sheet name="NUMERO DE YAPE" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="INTERBANK" sheetId="6" r:id="rId5"/>
+    <sheet name="PICHINCHA" sheetId="7" r:id="rId6"/>
+    <sheet name="BANBIF" sheetId="8" r:id="rId7"/>
+    <sheet name="NUMERO DE YAPE" sheetId="5" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">BANBIF!$B$1:$G$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">BBVA!$B$1:$G$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">BCP!$B$1:$G$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">FINANCIERO!$B$1:$G$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">INTERBANK!$B$1:$G$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">PICHINCHA!$B$1:$G$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">SCOTIABANK!$B$1:$G$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">BANBIF!$1:$2,BANBIF!$B:$G</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">BBVA!$1:$2,BBVA!$B:$G</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">BCP!$1:$2,BCP!$B:$G</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">FINANCIERO!$1:$2,FINANCIERO!$B:$G</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">INTERBANK!$1:$2,INTERBANK!$B:$G</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">PICHINCHA!$1:$2,PICHINCHA!$B:$G</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">SCOTIABANK!$1:$2,SCOTIABANK!$B:$G</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -50,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="20">
   <si>
     <t>TABLA DE PASAJES  - BBVA</t>
   </si>
@@ -104,6 +113,12 @@
   </si>
   <si>
     <t>Kevin Tavara Alama</t>
+  </si>
+  <si>
+    <t>TABLA DE PASAJES  - INTERBANK</t>
+  </si>
+  <si>
+    <t>TABLA DE PASAJES  - PICHINCHA</t>
   </si>
 </sst>
 </file>
@@ -451,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -491,6 +506,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -501,38 +517,38 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -848,6 +864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="B1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -861,14 +878,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
@@ -907,13 +924,13 @@
       <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="10"/>
     </row>
   </sheetData>
@@ -928,6 +945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Hoja2"/>
   <dimension ref="B1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -941,14 +959,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
@@ -971,29 +989,29 @@
       </c>
     </row>
     <row r="3" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="32"/>
+      <c r="B3" s="24"/>
       <c r="C3" s="13"/>
       <c r="D3" s="14"/>
       <c r="E3" s="13"/>
       <c r="F3" s="15"/>
-      <c r="G3" s="34"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
+      <c r="B4" s="25"/>
       <c r="C4" s="13"/>
       <c r="D4" s="14"/>
       <c r="E4" s="13"/>
       <c r="F4" s="15"/>
-      <c r="G4" s="35"/>
+      <c r="G4" s="27"/>
     </row>
     <row r="5" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="10"/>
     </row>
   </sheetData>
@@ -1010,6 +1028,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Hoja3"/>
   <dimension ref="B1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1023,14 +1042,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
@@ -1053,37 +1072,37 @@
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="32"/>
+      <c r="B3" s="24"/>
       <c r="C3" s="13"/>
       <c r="D3" s="14"/>
       <c r="E3" s="13"/>
       <c r="F3" s="15"/>
-      <c r="G3" s="34"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="33"/>
+      <c r="B4" s="25"/>
       <c r="C4" s="13"/>
       <c r="D4" s="14"/>
       <c r="E4" s="13"/>
       <c r="F4" s="15"/>
-      <c r="G4" s="35"/>
+      <c r="G4" s="27"/>
     </row>
     <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="10"/>
     </row>
     <row r="6" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1100,6 +1119,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Hoja4"/>
   <dimension ref="B1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1113,14 +1133,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
@@ -1159,13 +1179,13 @@
       <c r="G4" s="16"/>
     </row>
     <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="10"/>
     </row>
   </sheetData>
@@ -1179,7 +1199,254 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4D5FBC0-A493-4C10-8F70-D92E89C61EA7}">
+  <sheetPr codeName="Hoja5"/>
+  <dimension ref="B1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" style="17" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="11" style="17" customWidth="1"/>
+    <col min="4" max="4" width="56.85546875" style="17" customWidth="1"/>
+    <col min="5" max="5" width="18" style="17" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="17" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="16"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="16"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="16"/>
+    </row>
+    <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B5:F5"/>
+  </mergeCells>
+  <pageMargins left="0.11811023622047249" right="0.11811023622047249" top="0.27559055118110237" bottom="0.11811023622047249" header="0.19685039370078741" footer="0.15748031496062989"/>
+  <pageSetup scale="90" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A624EC1F-4C02-4D96-8294-F16DA016F51D}">
+  <sheetPr codeName="Hoja6"/>
+  <dimension ref="B1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" style="17" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="11" style="17" customWidth="1"/>
+    <col min="4" max="4" width="56.85546875" style="17" customWidth="1"/>
+    <col min="5" max="5" width="18" style="17" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="17" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="16"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="16"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="16"/>
+    </row>
+    <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B5:F5"/>
+  </mergeCells>
+  <pageMargins left="0.11811023622047249" right="0.11811023622047249" top="0.27559055118110237" bottom="0.11811023622047249" header="0.19685039370078741" footer="0.15748031496062989"/>
+  <pageSetup scale="90" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B916D9F8-38F2-40C6-8749-6AE530307F1B}">
+  <sheetPr codeName="Hoja8"/>
+  <dimension ref="B1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" style="17" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="11" style="17" customWidth="1"/>
+    <col min="4" max="4" width="56.85546875" style="17" customWidth="1"/>
+    <col min="5" max="5" width="18" style="17" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" style="17" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="2:7" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="16"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="16"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="16"/>
+    </row>
+    <row r="5" spans="2:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B5:F5"/>
+  </mergeCells>
+  <pageMargins left="0.11811023622047249" right="0.11811023622047249" top="0.27559055118110237" bottom="0.11811023622047249" header="0.19685039370078741" footer="0.15748031496062989"/>
+  <pageSetup scale="90" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr codeName="Hoja7"/>
   <dimension ref="B9:I29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1188,82 +1455,82 @@
   <sheetData>
     <row r="9" spans="8:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="19"/>
+      <c r="I10" s="20"/>
     </row>
     <row r="11" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H11" s="28">
+      <c r="H11" s="36">
         <v>917906797</v>
       </c>
-      <c r="I11" s="27"/>
+      <c r="I11" s="30"/>
     </row>
     <row r="12" spans="8:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="29" t="s">
+      <c r="H12" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="30"/>
+      <c r="I12" s="32"/>
     </row>
     <row r="16" spans="8:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="H17" s="25" t="s">
+      <c r="C17" s="20"/>
+      <c r="H17" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="I17" s="19"/>
+      <c r="I17" s="20"/>
     </row>
     <row r="18" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="28">
+      <c r="B18" s="36">
         <v>971340543</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="H18" s="26">
+      <c r="C18" s="30"/>
+      <c r="H18" s="29">
         <v>938503908</v>
       </c>
-      <c r="I18" s="27"/>
+      <c r="I18" s="30"/>
     </row>
     <row r="19" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="30"/>
+      <c r="C19" s="32"/>
       <c r="H19" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="I19" s="30"/>
+      <c r="I19" s="32"/>
     </row>
     <row r="21" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="E22" s="25" t="s">
+      <c r="C22" s="20"/>
+      <c r="E22" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="19"/>
-      <c r="H22" s="25" t="s">
+      <c r="F22" s="20"/>
+      <c r="H22" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="I22" s="19"/>
+      <c r="I22" s="20"/>
     </row>
     <row r="23" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="26">
+      <c r="B23" s="29">
         <v>980839245</v>
       </c>
-      <c r="C23" s="27"/>
-      <c r="E23" s="26">
+      <c r="C23" s="30"/>
+      <c r="E23" s="29">
         <v>996158270</v>
       </c>
-      <c r="F23" s="27"/>
-      <c r="H23" s="26">
+      <c r="F23" s="30"/>
+      <c r="H23" s="29">
         <v>931232818</v>
       </c>
-      <c r="I23" s="27"/>
+      <c r="I23" s="30"/>
     </row>
     <row r="24" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="6" t="s">
@@ -1273,24 +1540,24 @@
       <c r="E24" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="30"/>
+      <c r="F24" s="32"/>
       <c r="H24" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="I24" s="30"/>
+      <c r="I24" s="32"/>
     </row>
     <row r="26" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="19"/>
+      <c r="C27" s="20"/>
     </row>
     <row r="28" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="26">
+      <c r="B28" s="29">
         <v>933861787</v>
       </c>
-      <c r="C28" s="27"/>
+      <c r="C28" s="30"/>
     </row>
     <row r="29" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="11" t="s">
@@ -1300,15 +1567,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="E24:F24"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="E23:F23"/>
@@ -1319,6 +1577,15 @@
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="E24:F24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>